<commit_message>
Refactored documentation, and updated technical references
</commit_message>
<xml_diff>
--- a/students/alex-sample/input/student profile input.xlsx
+++ b/students/alex-sample/input/student profile input.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10703"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/I845765/Documents/college-finder/students/alex-sample/input/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/I845765/Documents/college-compass/students/alex-sample/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C737BB-BC41-314B-8BCE-A98FB94B117F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A2D78A-63C4-C540-A71F-785E23178F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Student Profile" sheetId="1" r:id="rId1"/>
@@ -661,9 +661,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="81">
   <si>
-    <t>College Finder — Student Profile Input</t>
-  </si>
-  <si>
     <t>Fill REQUIRED fields (yellow). Save this file in input/. Add transcript.pdf, resume.pdf, or test reports in the same folder when helpful.</t>
   </si>
   <si>
@@ -902,6 +899,9 @@
   </si>
   <si>
     <t>Prefer schools with strong internship placement in finance or consulting.</t>
+  </si>
+  <si>
+    <t>College Compass — Student Profile Input</t>
   </si>
 </sst>
 </file>
@@ -1310,119 +1310,119 @@
   <sheetData>
     <row r="1" spans="1:2" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="B1" s="8"/>
     </row>
     <row r="2" spans="1:2" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="8"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="3"/>
     </row>
     <row r="5" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>5</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>7</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>9</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" s="5">
-        <v>30000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>14</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>20</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B15" s="3"/>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B16" s="6">
         <v>12</v>
@@ -1430,7 +1430,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B17" s="6">
         <v>2027</v>
@@ -1438,7 +1438,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B18" s="6">
         <v>3.45</v>
@@ -1446,7 +1446,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B19" s="6">
         <v>3.68</v>
@@ -1454,15 +1454,15 @@
     </row>
     <row r="20" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>27</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B21" s="6">
         <v>1180</v>
@@ -1470,7 +1470,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B22" s="6">
         <v>26</v>
@@ -1478,7 +1478,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B23" s="6">
         <v>25</v>
@@ -1486,7 +1486,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B24" s="6">
         <v>27</v>
@@ -1494,7 +1494,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B25" s="6">
         <v>26</v>
@@ -1502,7 +1502,7 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B26" s="6">
         <v>26</v>
@@ -1510,7 +1510,7 @@
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B27" s="6">
         <v>2</v>
@@ -1518,21 +1518,21 @@
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B28" s="3"/>
     </row>
     <row r="29" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
+        <v>36</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>37</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B30" s="6">
         <v>2026</v>
@@ -1540,184 +1540,184 @@
     </row>
     <row r="31" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
+        <v>39</v>
+      </c>
+      <c r="B31" s="6" t="s">
         <v>40</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B32" s="3"/>
     </row>
     <row r="33" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" s="6" t="s">
         <v>43</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
+        <v>44</v>
+      </c>
+      <c r="B34" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B35" s="6"/>
     </row>
     <row r="36" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
+        <v>47</v>
+      </c>
+      <c r="B36" s="6" t="s">
         <v>48</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B37" s="6"/>
     </row>
     <row r="38" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
+        <v>51</v>
+      </c>
+      <c r="B39" s="6" t="s">
         <v>52</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B40" s="3"/>
     </row>
     <row r="41" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41" s="6" t="s">
         <v>55</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
+        <v>56</v>
+      </c>
+      <c r="B42" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
+        <v>58</v>
+      </c>
+      <c r="B43" s="6" t="s">
         <v>59</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
+        <v>60</v>
+      </c>
+      <c r="B44" s="6" t="s">
         <v>61</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
+        <v>62</v>
+      </c>
+      <c r="B45" s="6" t="s">
         <v>63</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
+        <v>65</v>
+      </c>
+      <c r="B47" s="6" t="s">
         <v>66</v>
-      </c>
-      <c r="B47" s="6" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
+        <v>67</v>
+      </c>
+      <c r="B48" s="6" t="s">
         <v>68</v>
-      </c>
-      <c r="B48" s="6" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
+        <v>69</v>
+      </c>
+      <c r="B49" s="6" t="s">
         <v>70</v>
-      </c>
-      <c r="B49" s="6" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B50" s="3"/>
     </row>
     <row r="51" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
+        <v>72</v>
+      </c>
+      <c r="B51" s="6" t="s">
         <v>73</v>
-      </c>
-      <c r="B51" s="6" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
+        <v>74</v>
+      </c>
+      <c r="B52" s="6" t="s">
         <v>75</v>
-      </c>
-      <c r="B52" s="6" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
+        <v>76</v>
+      </c>
+      <c r="B53" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="B53" s="6" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
+        <v>78</v>
+      </c>
+      <c r="B54" s="6" t="s">
         <v>79</v>
-      </c>
-      <c r="B54" s="6" t="s">
-        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>